<commit_message>
feat: Add global pricing adjustment configs, individual custom overrides, manual visibility toggle, clean laptop titles, rounded WhatsApp button, and daily scraper GitHub workflow
</commit_message>
<xml_diff>
--- a/precios_venta.xlsx
+++ b/precios_venta.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,7 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,6 +522,11 @@
           <t>Ganancia USD</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -560,6 +566,11 @@
       <c r="I2" s="4" t="n">
         <v>297.8</v>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -599,6 +610,11 @@
       <c r="I3" s="4" t="n">
         <v>389.8</v>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -638,6 +654,11 @@
       <c r="I4" s="4" t="n">
         <v>439.8</v>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -677,6 +698,11 @@
       <c r="I5" s="4" t="n">
         <v>469.8</v>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -716,6 +742,11 @@
       <c r="I6" s="4" t="n">
         <v>299.8</v>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -755,6 +786,11 @@
       <c r="I7" s="4" t="n">
         <v>509.8</v>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -794,6 +830,11 @@
       <c r="I8" s="4" t="n">
         <v>285.8</v>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -833,6 +874,11 @@
       <c r="I9" s="4" t="n">
         <v>319.8</v>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -872,6 +918,11 @@
       <c r="I10" s="4" t="n">
         <v>349.8</v>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -911,6 +962,11 @@
       <c r="I11" s="4" t="n">
         <v>359.8</v>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -950,6 +1006,11 @@
       <c r="I12" s="4" t="n">
         <v>519.8</v>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -989,6 +1050,11 @@
       <c r="I13" s="4" t="n">
         <v>339.8</v>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1028,6 +1094,11 @@
       <c r="I14" s="4" t="n">
         <v>319.8</v>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1067,6 +1138,11 @@
       <c r="I15" s="4" t="n">
         <v>479.8</v>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1106,6 +1182,11 @@
       <c r="I16" s="4" t="n">
         <v>579.8</v>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1145,6 +1226,11 @@
       <c r="I17" s="4" t="n">
         <v>399.8</v>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1184,6 +1270,11 @@
       <c r="I18" s="4" t="n">
         <v>313.8</v>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1223,6 +1314,11 @@
       <c r="I19" s="4" t="n">
         <v>799.8</v>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1262,6 +1358,11 @@
       <c r="I20" s="4" t="n">
         <v>335.8</v>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1301,6 +1402,11 @@
       <c r="I21" s="4" t="n">
         <v>419.8</v>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1315,7 +1421,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Notebook Dell Precision 7780 Intel Core i9 13950HX Tela Full HD 17.3" / 128GB de RAM / 4TB SSD / GeForce RTX5000A 16GB / Win11 Pro - Cinza (Inglês)</t>
+          <t>Notebook Dell Precision 7780 Intel Core i9-13950HX / 128GB RAM / 4TB SSD / GeForce RTX 5000 Ada 16GB / 17.3'' FHD IPS / Win11 Pro - Gris</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1340,6 +1446,11 @@
       <c r="I22" s="4" t="n">
         <v>1015.8</v>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1379,6 +1490,11 @@
       <c r="I23" s="4" t="n">
         <v>379.8</v>
       </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1418,6 +1534,11 @@
       <c r="I24" s="4" t="n">
         <v>419.8</v>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1457,6 +1578,11 @@
       <c r="I25" s="4" t="n">
         <v>329.8</v>
       </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1496,6 +1622,11 @@
       <c r="I26" s="4" t="n">
         <v>519.8</v>
       </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1535,6 +1666,11 @@
       <c r="I27" s="4" t="n">
         <v>319.8</v>
       </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1574,6 +1710,11 @@
       <c r="I28" s="4" t="n">
         <v>499.8</v>
       </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1613,6 +1754,11 @@
       <c r="I29" s="4" t="n">
         <v>339.8</v>
       </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1652,6 +1798,11 @@
       <c r="I30" s="4" t="n">
         <v>419.8</v>
       </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1691,6 +1842,11 @@
       <c r="I31" s="4" t="n">
         <v>539.8</v>
       </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1730,6 +1886,11 @@
       <c r="I32" s="4" t="n">
         <v>799.8</v>
       </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1769,6 +1930,11 @@
       <c r="I33" s="4" t="n">
         <v>539.8</v>
       </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1808,6 +1974,11 @@
       <c r="I34" s="4" t="n">
         <v>439.8</v>
       </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1847,6 +2018,11 @@
       <c r="I35" s="4" t="n">
         <v>579.8</v>
       </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1886,50 +2062,60 @@
       <c r="I36" s="4" t="n">
         <v>449.8</v>
       </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>54911</t>
+          <t>57717</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ASUS</t>
+          <t>Acer</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>PC Gamer Intel Core i7-14700F / 32GB RAM DDR5 / 1TB SSD NVMe / GeForce RTX 4070 12GB / WaterCooler 240mm - Negro</t>
+          <t>Notebook Acer GadGet E10 ETBook Yoga CWI557 Intel Core i3-1315U / 8GB RAM / 256GB SSD / 13.4'' Touch 2.5K / Win11 - Gris</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>office</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1699</v>
+        <v>469</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2178.8</v>
+        <v>702.8</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>3224624</v>
+        <v>1040144</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>479.8</v>
+        <v>233.8</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>54912</t>
+          <t>58300</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1939,163 +2125,183 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>PC Gamer AMD Ryzen 5 7600X / 16GB RAM DDR5 / 1TB SSD NVMe / GeForce RTX 4060 Ti 8GB - Negro</t>
+          <t>Notebook ASUS Vivobook Go 15 E1504FA AMD Ryzen 5 7520U / 8GB RAM / 512GB SSD / AMD Radeon 610M / 15.6'' FHD / Win11 - Negro</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>office</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>1149</v>
+        <v>419</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>1518.8</v>
+        <v>642.8</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>2247824</v>
+        <v>951344</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>369.8</v>
+        <v>223.8</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>54914</t>
+          <t>58280</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>ASUS</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>PC Gamer Extrema Intel Core i9-14900K / 64GB RAM DDR5 / 2TB SSD / GeForce RTX 4090 24GB / WaterCooler 360mm - Blanco</t>
+          <t>Notebook Lenovo IdeaPad 1 15IRU7 Intel Core i5-1335U / 8GB RAM / 512GB SSD / Intel Iris Xe / 15.6'' Touch FHD / Win11 - Gris</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>office</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>3799</v>
+        <v>519</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>4698.8</v>
+        <v>762.8</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>6954224</v>
+        <v>1128944</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>899.8</v>
+        <v>243.8</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>54916</t>
+          <t>58350</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>PC Workstation AMD Ryzen 9 7900X / 64GB RAM DDR5 / 2TB SSD / GeForce RTX 4080 Super 16GB - Negro</t>
+          <t>Notebook HP 15-FD0025WM AMD Ryzen 5 7520U / 8GB RAM / 1TB SSD / AMD Radeon 610M / 15.6'' Touch FHD / Win11 - Azul</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>productivity</t>
+          <t>office</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2499</v>
+        <v>479</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>3138.8</v>
+        <v>714.8</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>4645424</v>
+        <v>1057904</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>639.8</v>
+        <v>235.8</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>54918</t>
+          <t>58410</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>ASUS</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>PC Gamer Ryzen 7 5700X / 32GB RAM / 1TB SSD NVMe / GeForce RTX 4060 8GB / Cooler Tower - Negro</t>
+          <t>Notebook Dell Inspiron 15 3520 Intel Core i5-1235U / 16GB RAM / 512GB SSD / Intel Iris Xe / 15.6'' FHD 120Hz / Win11 - Carbon</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>office</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>999</v>
+        <v>549</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>1338.8</v>
+        <v>798.8</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1981424</v>
+        <v>1182224</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>339.8</v>
+        <v>249.8</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>54919</t>
+          <t>58490</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>ASUS</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Apple Mac Mini Apple M3 Chip (8-Core CPU / 10-Core GPU) / 16GB RAM / 512GB SSD - Plateado</t>
+          <t>Notebook ASUS Vivobook 16 M1605YA AMD Ryzen 7 7730U / 16GB RAM / 1TB SSD / AMD Radeon Graphics / 16'' WUXGA IPS / Win11 - Plata</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2105,20 +2311,201 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>899</v>
+        <v>679</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>1218.8</v>
+        <v>954.8</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>1803824</v>
+        <v>1413104</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>319.8</v>
+        <v>275.8</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>58510</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Acer</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Notebook Acer Aspire 5 A515-58P Intel Core i5-1335U / 8GB RAM / 512GB SSD / Intel UHD Graphics / 15.6'' FHD / Win11 - Gris</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>notebook</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>489</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>726.8</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>1075664</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>237.8</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>58620</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Notebook HP 15-FC0015TG AMD Ryzen 3 7320U / 8GB RAM / 256GB SSD / AMD Radeon 610M / 15.6'' HD / Win11 S - Gris</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>notebook</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>329</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>534.8</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>791504</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>205.8</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>58701</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Lenovo</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Notebook Lenovo IdeaPad Slim 3 15IAN8 Intel Core i3-N305 / 8GB RAM / 256GB SSD / 15.6'' FHD / Win11 - Azul</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>notebook</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>369</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>582.8</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>862544</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>213.8</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>59301</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Notebook Dell Inspiron 15 3530 Intel Core i3-1305U / 8GB RAM / 512GB SSD / Intel UHD Graphics / 15.6'' Touch FHD / Win11 - Carbon</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>office</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>notebook</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>459</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>690.8</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>1022384</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>231.8</v>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>